<commit_message>
Update Excel templates and modify person_class.py for product handling; remove unused files and enhance test script.
</commit_message>
<xml_diff>
--- a/bestilling_sporsmal.xlsx
+++ b/bestilling_sporsmal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/NTNUI-klubbklar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_AD4D1D646341095ACB7000D2C594FF4C683EDF15" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD2965EB-9320-470B-905C-6DE627A6B8FA}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_AD4D1D646341095ACB7000D2C594FF4C683EDF15" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADBE5903-E85D-46AC-A86E-43181D8006B3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>product</t>
   </si>
@@ -36,26 +36,80 @@
     <t>type</t>
   </si>
   <si>
-    <t>float/bool/int/str</t>
-  </si>
-  <si>
     <t>thing</t>
   </si>
   <si>
-    <t>size/amount</t>
-  </si>
-  <si>
-    <t>bool-true</t>
+    <t>str</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>Size of t-shirt(s)</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>bool-false</t>
+  </si>
+  <si>
+    <t>skal ikke ha</t>
+  </si>
+  <si>
+    <t>Amount of black t-shirts</t>
+  </si>
+  <si>
+    <t>Amount of red t-shirts</t>
+  </si>
+  <si>
+    <t>Amount of white t-shirts</t>
+  </si>
+  <si>
+    <t>If yes, what should be printed on the back?</t>
+  </si>
+  <si>
+    <t>Comments regarding the t-shirt order.</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>Tskjorte</t>
+  </si>
+  <si>
+    <t>color</t>
+  </si>
+  <si>
+    <t>Sort</t>
+  </si>
+  <si>
+    <t>Rød</t>
+  </si>
+  <si>
+    <t>Hvit</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -81,8 +135,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -363,13 +420,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -380,18 +441,110 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>